<commit_message>
Fix track_nelly_aov.py: update stale price selector (KNOWN_ISSUES #6)
Nelly's frontend rebuild renamed the price span's class from
"text-sm text-darkGrey" to "text-subhead leading-none text-darkGrey",
so fetch_prices() found 0 prices on all 10 pages since 2026-07-20 and
silently exited without writing (no Excel row, no DB row).

Confirmed live via Selenium DOM inspection: the old discount-vs-regular
price split (<ins> for sale price, <del> for original) no longer exists
either - the listing page now shows exactly one price per product card -
so removed that now-unnecessary logic along with the dead selector.

Verified end-to-end: all 10 pages returned 32 prices each (320 total),
median 349 kr / mean 423.41 kr for 2026-08-05, a plausible mean>median
skew consistent with pre-breakage history. Row written to both
data/nelly_aov.xlsx and the nelly_aov table.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/nelly_aov.xlsx
+++ b/data/nelly_aov.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C292"/>
+  <dimension ref="A1:C293"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10.1640625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -4218,6 +4218,19 @@
         <v>301</v>
       </c>
     </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B293" t="n">
+        <v>349</v>
+      </c>
+      <c r="C293" t="n">
+        <v>423.41</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>